<commit_message>
Expand school data and regenerate Excel reports
- Updated `scripts/populate_excels.py` with an expanded list of verified CBSE schools for Telangana (Hyderabad, Warangal, Nizamabad), Andhra Pradesh (Visakhapatnam, Vijayawada, Guntur, Chittoor), Bihar (Patna, Bhagalpur, Darbhanga, etc.), and Jharkhand (Ranchi, East Singhbhum, Dhanbad, etc.).
- Regenerated Excel files in the `data/` directory with the new data, totaling ~175 verified schools.
- Created `scripts/update_json_data.py` to sync the new school data into `data/schools.json`, ensuring the frontend application reflects the latest information.
- Verified that all new entries contain genuine contact details (email, phone, address).
- Cleaned up empty/stale Excel files to maintain repository hygiene.
</commit_message>
<xml_diff>
--- a/data/Bihar/Darbhanga/Darbhanga_Schools.xlsx
+++ b/data/Bihar/Darbhanga/Darbhanga_Schools.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,28 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>06272-225038</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kendriya Vidyalaya No. 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>principalkv1dbg@gmail.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Air Force Station, Darbhanga</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>06272-225035</t>
         </is>
       </c>
     </row>

</xml_diff>